<commit_message>
MGA reporting: any company, any bore, any assessment stage; access and security note
All ten tenure holders in the UWIR 2025 tenure layer can report, plus "Other" with a typed
company name in email mode; registers list the extra companies switched off until OGIA issues
codes. The bore check no longer treats bores outside the Surat CMA or off the IAA list as
mistakes: any bore with a make good obligation can be reported. New MGA_ACCESS_AND_SECURITY.md
explains who can submit, who can see what and what a personal log-in option would need.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SUXuRFEjE9pVDU2NswBRex
</commit_message>
<xml_diff>
--- a/bore_search_tool/power_automate/MGA_master_register.xlsx
+++ b/bore_search_tool/power_automate/MGA_master_register.xlsx
@@ -178,8 +178,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TenureHolders" displayName="TenureHolders" ref="A1:F5" headerRowCount="1">
-  <autoFilter ref="A1:F5"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TenureHolders" displayName="TenureHolders" ref="A1:F11" headerRowCount="1">
+  <autoFilter ref="A1:F11"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Code"/>
     <tableColumn id="2" name="HolderName"/>
@@ -786,7 +786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -939,6 +939,174 @@
       <c r="E5" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SENEX</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Senex Energy</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>SET-BY-OGIA-SENEX</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Not yet onboarded: fill AccessCode and EmailDomain, then set Active to Yes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AGL</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>AGL</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>SET-BY-OGIA-AGL</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Not yet onboarded: fill AccessCode and EmailDomain, then set Active to Yes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ADZ ENERGY</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ADZ Energy</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>SET-BY-OGIA-ADZ-ENERGY</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Not yet onboarded: fill AccessCode and EmailDomain, then set Active to Yes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BRIDGEPORT ENERGY</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Bridgeport Energy</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>SET-BY-OGIA-BRIDGEPORT-ENERGY</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Not yet onboarded: fill AccessCode and EmailDomain, then set Active to Yes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DENISON GAS</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Denison Gas</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>SET-BY-OGIA-DENISON-GAS</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Not yet onboarded: fill AccessCode and EmailDomain, then set Active to Yes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>OGT</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>OGT</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>SET-BY-OGIA-OGT</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Not yet onboarded: fill AccessCode and EmailDomain, then set Active to Yes.</t>
         </is>
       </c>
     </row>

</xml_diff>